<commit_message>
finished leaderboard, fixed up some documentation files also
</commit_message>
<xml_diff>
--- a/presentations/sprintbacklog6.xlsx
+++ b/presentations/sprintbacklog6.xlsx
@@ -5,11 +5,11 @@
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yathanvidyananthan/Desktop/cscc01/L01_03/presentations/links/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yathanvidyananthan/Desktop/cscc01/L01_03/presentations/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="28800" windowHeight="16980"/>
+    <workbookView xWindow="-20" yWindow="460" windowWidth="28800" windowHeight="16980"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Plan and Sprint Report" sheetId="5" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="46">
   <si>
     <t>Task</t>
   </si>
@@ -137,6 +137,36 @@
   </si>
   <si>
     <t>clean up existing assignments and questions and make 1 or 2 good assignments for demo purposes</t>
+  </si>
+  <si>
+    <t>As Edward Squid (student), I would like be able to see a leaderboard with a list of top students with the highest scores</t>
+  </si>
+  <si>
+    <t>set up backend to return top 3 students with their average</t>
+  </si>
+  <si>
+    <t>using djanga set up new tables, to properly calculate average and return to front end</t>
+  </si>
+  <si>
+    <t>set up frontend to receive top 3 students with a nice leaderboard</t>
+  </si>
+  <si>
+    <t>use css make the leadboard look attractive on the welcome.html page</t>
+  </si>
+  <si>
+    <t>As Sohee Kang (professor), I need to create accounts for students and TA's' so that they can access quizzes remotely</t>
+  </si>
+  <si>
+    <t>set up frontend to allow for text and excel files for student account creation</t>
+  </si>
+  <si>
+    <t>set up backend to read this file and create accounts for these studeents</t>
+  </si>
+  <si>
+    <t>read the files on python using py librariers, and insert the students username and password into the correct table</t>
+  </si>
+  <si>
+    <t>use html forms to allow for a file upload</t>
   </si>
 </sst>
 </file>
@@ -248,7 +278,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -269,15 +299,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -285,6 +306,18 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -542,25 +575,25 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10.0</c:v>
+                  <c:v>17.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>10.0</c:v>
+                  <c:v>17.0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>10.0</c:v>
+                  <c:v>14.0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.0</c:v>
+                  <c:v>2.0</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.0</c:v>
@@ -706,28 +739,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>15.0</c:v>
+                  <c:v>22.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -750,11 +783,11 @@
         </c:dLbls>
         <c:marker val="1"/>
         <c:smooth val="0"/>
-        <c:axId val="-808417808"/>
-        <c:axId val="-808372800"/>
+        <c:axId val="-219979632"/>
+        <c:axId val="-386161456"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="-808417808"/>
+        <c:axId val="-219979632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -853,7 +886,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-808372800"/>
+        <c:crossAx val="-386161456"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -861,7 +894,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="-808372800"/>
+        <c:axId val="-386161456"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -980,7 +1013,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="-808417808"/>
+        <c:crossAx val="-219979632"/>
         <c:crossesAt val="1.0"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1710,7 +1743,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000003000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2016,7 +2049,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z12"/>
+  <dimension ref="A1:Z16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.1640625" style="1" customWidth="1"/>
@@ -2027,13 +2060,13 @@
     <col min="7" max="7" width="8.33203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="2.83203125" style="3" customWidth="1"/>
     <col min="9" max="9" width="13.5" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" style="12" customWidth="1"/>
+    <col min="10" max="10" width="14.5" style="13" customWidth="1"/>
     <col min="11" max="11" width="5.83203125" style="1" customWidth="1"/>
     <col min="12" max="13" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="6" style="1" customWidth="1"/>
     <col min="17" max="17" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.6640625" style="10" customWidth="1"/>
-    <col min="19" max="19" width="7" style="11" customWidth="1"/>
+    <col min="18" max="18" width="3.6640625" style="3" customWidth="1"/>
+    <col min="19" max="19" width="7" style="14" customWidth="1"/>
     <col min="20" max="26" width="6" style="1" customWidth="1"/>
     <col min="27" max="16384" width="12" style="1"/>
   </cols>
@@ -2063,7 +2096,7 @@
       <c r="I1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="13" t="s">
         <v>11</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -2087,7 +2120,7 @@
       <c r="Q1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="S1" s="14" t="s">
         <v>12</v>
       </c>
       <c r="T1" s="3" t="s">
@@ -2116,7 +2149,7 @@
       <c r="A2" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="13"/>
+      <c r="B2" s="10"/>
       <c r="C2" s="5">
         <v>1</v>
       </c>
@@ -2138,7 +2171,7 @@
     </row>
     <row r="3" spans="1:26" ht="47" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="9"/>
-      <c r="B3" s="13"/>
+      <c r="B3" s="10"/>
       <c r="C3" s="5">
         <v>2</v>
       </c>
@@ -2160,7 +2193,7 @@
     </row>
     <row r="4" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="9"/>
-      <c r="B4" s="13"/>
+      <c r="B4" s="10"/>
       <c r="C4" s="4">
         <v>3</v>
       </c>
@@ -2182,7 +2215,7 @@
     </row>
     <row r="5" spans="1:26" ht="29" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="9"/>
-      <c r="B5" s="13"/>
+      <c r="B5" s="10"/>
       <c r="C5" s="5">
         <v>4</v>
       </c>
@@ -2202,98 +2235,198 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="7" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B7" s="5"/>
+    <row r="6" spans="1:26" ht="40" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A6" s="16">
+        <v>14</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="4">
+        <v>5</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" s="1">
+        <v>2</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="P6" s="1">
+        <v>2</v>
+      </c>
     </row>
-    <row r="8" spans="1:26" ht="15" x14ac:dyDescent="0.2">
-      <c r="B8" s="5"/>
-      <c r="G8" s="2">
-        <f>SUM(G2:G5)</f>
-        <v>15</v>
-      </c>
-      <c r="K8" s="6">
-        <f>SUM(K1:K5)</f>
+    <row r="7" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A7" s="16"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="5">
+        <v>6</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" s="1">
+        <v>2</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A8" s="16">
+        <v>1</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="5">
+        <v>7</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="O8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="28" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A9" s="16"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="5">
+        <v>8</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="1">
+        <v>2</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="O9" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="18" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+    </row>
+    <row r="11" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B11" s="5"/>
+    </row>
+    <row r="12" spans="1:26" ht="15" x14ac:dyDescent="0.2">
+      <c r="B12" s="5"/>
+      <c r="G12" s="2">
+        <f>SUM(G2:G9)</f>
+        <v>22</v>
+      </c>
+      <c r="K12" s="6">
+        <f>SUM(K2:K9)</f>
         <v>0</v>
       </c>
-      <c r="L8" s="6">
-        <f>SUM(L2:L5)</f>
+      <c r="L12" s="6">
+        <f t="shared" ref="L12:Q12" si="0">SUM(L2:L9)</f>
         <v>0</v>
       </c>
-      <c r="M8" s="6">
-        <f>SUM(M2:M5)</f>
+      <c r="M12" s="6">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="N8" s="6">
-        <f>SUM(N2:N5)</f>
-        <v>0</v>
-      </c>
-      <c r="O8" s="6">
-        <f>SUM(O2:O5)</f>
-        <v>0</v>
-      </c>
-      <c r="P8" s="6">
-        <f>SUM(P2:P5)</f>
-        <v>10</v>
-      </c>
-      <c r="Q8" s="6">
-        <f>SUM(Q2:Q5)</f>
-        <v>0</v>
-      </c>
-      <c r="T8" s="2">
-        <f t="shared" ref="T8:Z8" si="0">SUM(T2:T7)</f>
-        <v>0</v>
-      </c>
-      <c r="U8" s="2">
+      <c r="N12" s="6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="V8" s="2">
+      <c r="O12" s="6">
         <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="P12" s="6">
+        <f>SUM(P2:P9)</f>
+        <v>12</v>
+      </c>
+      <c r="Q12" s="6">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="T12" s="2">
+        <f t="shared" ref="T12:Z12" si="1">SUM(T2:T11)</f>
         <v>0</v>
       </c>
-      <c r="W8" s="2">
-        <f t="shared" si="0"/>
+      <c r="U12" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="X8" s="2">
-        <f t="shared" si="0"/>
+      <c r="V12" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Y8" s="2">
-        <f t="shared" si="0"/>
+      <c r="W12" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Z8" s="2">
-        <f t="shared" si="0"/>
+      <c r="X12" s="2">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="Y12" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Z12" s="2">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="Z9" s="2"/>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.15">
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="Z13" s="2"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="T10" s="2"/>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="2"/>
-      <c r="Y10" s="2"/>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.15">
+      <c r="T14" s="2"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="2"/>
+      <c r="W14" s="2"/>
+      <c r="X14" s="2"/>
+      <c r="Y14" s="2"/>
     </row>
-    <row r="12" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="16" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15"/>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="R1:R1048576"/>
-    <mergeCell ref="S1:S1048576"/>
-    <mergeCell ref="J1:J1048576"/>
+  <mergeCells count="6">
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="B2:B5"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A8:A9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2312,17 +2445,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -2358,29 +2491,31 @@
         <v>8</v>
       </c>
       <c r="B3">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C3">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D3">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E3">
-        <f>15-5</f>
-        <v>10</v>
+        <f>22-5</f>
+        <v>17</v>
       </c>
       <c r="F3">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G3">
-        <v>10</v>
+        <f>17-3</f>
+        <v>14</v>
       </c>
       <c r="H3">
-        <f>10-10</f>
-        <v>0</v>
+        <f>14-12</f>
+        <v>2</v>
       </c>
       <c r="I3">
+        <f>2-2</f>
         <v>0</v>
       </c>
     </row>
@@ -2389,40 +2524,40 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="F4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I4">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>